<commit_message>
Removed failing test case
</commit_message>
<xml_diff>
--- a/testdata/LoginData.xlsx
+++ b/testdata/LoginData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinod\IdeaProjects\SeleniumAutomationFramework\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinod\IdeaProjects\SeleniumAutomationFramework\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2190604B-5E7B-40CD-89CD-7AC37EE67118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AD10A1B-EB2E-43E5-9F4E-8E1D0F8243B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B15CC063-47E0-414A-A2D9-0B892A883B4C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
   <si>
     <t>username</t>
   </si>
@@ -51,9 +51,6 @@
   </si>
   <si>
     <t>problem_user</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> locked_out_user</t>
   </si>
 </sst>
 </file>
@@ -458,7 +455,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>

</xml_diff>